<commit_message>
v7 print pack: seven exhibits rendered from workbook values; evaluator; verification workflow script
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014kuv7KAQpTthYpd1CUvsfc
</commit_message>
<xml_diff>
--- a/outputs/JSW_R2_workbook_v7.xlsx
+++ b/outputs/JSW_R2_workbook_v7.xlsx
@@ -9921,7 +9921,7 @@
         </is>
       </c>
       <c r="C118" s="6" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
@@ -9935,7 +9935,7 @@
       </c>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Assumption; must sit below the human cost per call (Rs 8 to 25) for the buyer to save</t>
         </is>
       </c>
       <c r="G118" s="4" t="inlineStr"/>
@@ -9956,10 +9956,10 @@
         </is>
       </c>
       <c r="L118" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M118" s="6" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="N118" s="4" t="inlineStr"/>
     </row>
@@ -13821,7 +13821,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10 to 20</t>
+          <t>5 to 12</t>
         </is>
       </c>
     </row>
@@ -17559,7 +17559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -17881,7 +17881,7 @@
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>The buyer's saving</t>
+          <t>Under 1 means the buyer saves; India's cheap human calls leave a thin price room</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -17890,11 +17890,11 @@
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Intercom Fin per resolution, in rupees</t>
+          <t>Buyer's saving per call</t>
         </is>
       </c>
       <c r="B19" s="11">
-        <f>in_A9*in_A7</f>
+        <f>B8-B16</f>
         <v/>
       </c>
       <c r="C19" t="inlineStr">
@@ -17903,21 +17903,17 @@
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr"/>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>A9, A7</t>
-        </is>
-      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" s="1" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Agentforce per conversation, in rupees</t>
+          <t>Intercom Fin per resolution, in rupees</t>
         </is>
       </c>
       <c r="B20" s="11">
-        <f>in_A10*in_A7</f>
+        <f>in_A9*in_A7</f>
         <v/>
       </c>
       <c r="C20" t="inlineStr">
@@ -17928,7 +17924,7 @@
       <c r="D20" s="1" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>A10, A7</t>
+          <t>A9, A7</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr"/>
@@ -17936,22 +17932,22 @@
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Exception staff threshold (share of revenue)</t>
-        </is>
-      </c>
-      <c r="B21" s="12">
-        <f>in_A37</f>
+          <t>Agentforce per conversation, in rupees</t>
+        </is>
+      </c>
+      <c r="B21" s="11">
+        <f>in_A10*in_A7</f>
         <v/>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>INR</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>A37</t>
+          <t>A10, A7</t>
         </is>
       </c>
       <c r="F21" s="1" t="inlineStr"/>
@@ -17959,11 +17955,11 @@
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
-          <t>Stellaris: share of 216 voice AI companies targeting existing spend</t>
+          <t>Exception staff threshold (share of revenue)</t>
         </is>
       </c>
       <c r="B22" s="12">
-        <f>in_A14</f>
+        <f>in_A37</f>
         <v/>
       </c>
       <c r="C22" t="inlineStr">
@@ -17974,10 +17970,33 @@
       <c r="D22" s="1" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
+          <t>A37</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Stellaris: share of 216 voice AI companies targeting existing spend</t>
+        </is>
+      </c>
+      <c r="B23" s="12">
+        <f>in_A14</f>
+        <v/>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
           <t>A14</t>
         </is>
       </c>
-      <c r="F22" s="1" t="inlineStr"/>
+      <c r="F23" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>